<commit_message>
Add Hararghe-specific options to water source and coping action choice lists
</commit_message>
<xml_diff>
--- a/form/hararghe_hna_v1.xlsx
+++ b/form/hararghe_hna_v1.xlsx
@@ -4192,7 +4192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E119"/>
+  <dimension ref="A1:E126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6751,6 +6751,139 @@
       </c>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>water_src</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>birka</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Traditional pond (birka)</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>water_src</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>shallow_well</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Shallow well</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>water_src</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>motorised_borehole</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Motorised borehole</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>water_src</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>tanker</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Water tanker</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>coping_actions</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>sold_livestock</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Sold livestock</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>coping_actions</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>food_aid</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Received food aid</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>coping_actions</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>cash_assistance</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Received cash assistance</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>